<commit_message>
Adds Tour Export Adds Tour Import
</commit_message>
<xml_diff>
--- a/documentation/reports/checklist.xlsx
+++ b/documentation/reports/checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="67">
   <si>
     <t xml:space="preserve">Checklist Tourplanner Exam - Final Hand-In</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t xml:space="preserve">Export tour data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">backend implemented</t>
   </si>
   <si>
     <t xml:space="preserve">Import tour data</t>
@@ -693,7 +696,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.63"/>
@@ -1014,20 +1017,26 @@
         <v>2</v>
       </c>
       <c r="D47" s="12"/>
+      <c r="F47" s="0" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D48" s="12"/>
+      <c r="F48" s="0" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="50" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C50" s="7" t="n">
         <v>2</v>
@@ -1036,12 +1045,12 @@
     </row>
     <row r="52" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C53" s="7" t="n">
         <v>2</v>
@@ -1050,7 +1059,7 @@
     </row>
     <row r="54" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C54" s="7" t="n">
         <v>1</v>
@@ -1059,7 +1068,7 @@
     </row>
     <row r="55" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C55" s="7" t="n">
         <v>2</v>
@@ -1068,7 +1077,7 @@
     </row>
     <row r="56" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C56" s="7" t="n">
         <v>2</v>
@@ -1077,7 +1086,7 @@
     </row>
     <row r="57" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C57" s="7" t="n">
         <v>2</v>
@@ -1086,7 +1095,7 @@
     </row>
     <row r="58" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>1</v>
@@ -1095,7 +1104,7 @@
     </row>
     <row r="59" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C59" s="7" t="n">
         <v>1</v>
@@ -1104,7 +1113,7 @@
     </row>
     <row r="60" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C60" s="7" t="n">
         <v>1</v>
@@ -1113,7 +1122,7 @@
     </row>
     <row r="63" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -1121,7 +1130,7 @@
     </row>
     <row r="64" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>3</v>
@@ -1130,7 +1139,7 @@
     </row>
     <row r="65" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C65" s="7" t="n">
         <v>1</v>
@@ -1139,7 +1148,7 @@
     </row>
     <row r="66" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B66" s="9"/>
       <c r="C66" s="7"/>
@@ -1147,7 +1156,7 @@
     </row>
     <row r="67" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C67" s="7" t="n">
         <v>1</v>
@@ -1156,7 +1165,7 @@
     </row>
     <row r="68" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>1</v>
@@ -1165,7 +1174,7 @@
     </row>
     <row r="69" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C69" s="7" t="n">
         <v>1</v>
@@ -1174,7 +1183,7 @@
     </row>
     <row r="70" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>1</v>
@@ -1183,7 +1192,7 @@
     </row>
     <row r="71" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C71" s="7" t="n">
         <v>0.5</v>
@@ -1192,7 +1201,7 @@
     </row>
     <row r="72" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C72" s="7" t="n">
         <v>0.5</v>
@@ -1201,14 +1210,14 @@
     </row>
     <row r="74" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
     </row>
     <row r="76" s="15" customFormat="true" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B76" s="15" t="n">
         <f aca="false">IF(MIN(B9:B19)=1,SUM(B25:B74),0)</f>

</xml_diff>

<commit_message>
Adds Tour CRUD Integrates Tour CRUD
</commit_message>
<xml_diff>
--- a/documentation/reports/checklist.xlsx
+++ b/documentation/reports/checklist.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="71">
   <si>
     <t xml:space="preserve">Checklist Tourplanner Exam - Final Hand-In</t>
   </si>
@@ -94,9 +94,24 @@
     <t xml:space="preserve">GUI in general</t>
   </si>
   <si>
+    <t xml:space="preserve">Frontend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F. Impl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. Impl</t>
+  </si>
+  <si>
     <t xml:space="preserve">Correct data binding between UI elements and view model properties</t>
   </si>
   <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
     <t xml:space="preserve">UI responds to window size changes</t>
   </si>
   <si>
@@ -149,9 +164,6 @@
   </si>
   <si>
     <t xml:space="preserve">Export tour data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">backend implemented</t>
   </si>
   <si>
     <t xml:space="preserve">Import tour data</t>
@@ -524,34 +536,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -696,7 +708,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.63"/>
@@ -853,39 +865,78 @@
       <c r="A24" s="6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
-    </row>
-    <row r="26" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
-    </row>
-    <row r="27" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E26" s="6"/>
+      <c r="F26" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+    </row>
+    <row r="27" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
-    </row>
-    <row r="29" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E27" s="1"/>
+      <c r="F27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G27" s="0"/>
+      <c r="H27" s="0"/>
+      <c r="I27" s="0"/>
+    </row>
+    <row r="29" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="10" t="n">
@@ -894,18 +945,30 @@
       <c r="D30" s="10" t="n">
         <v>2</v>
       </c>
+      <c r="F30" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
+      <c r="F31" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12" t="n">
@@ -913,12 +976,15 @@
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="12" t="n">
@@ -926,185 +992,298 @@
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
       <c r="E34" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D37" s="12"/>
+      <c r="F37" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B38" s="9"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
+      <c r="G38" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="7"/>
-    </row>
-    <row r="40" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F39" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-    </row>
-    <row r="42" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E40" s="1"/>
+      <c r="F40" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G40" s="0"/>
+      <c r="H40" s="0"/>
+      <c r="I40" s="0"/>
+    </row>
+    <row r="42" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>38</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C43" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D43" s="7"/>
-    </row>
-    <row r="44" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F43" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B44" s="1"/>
       <c r="C44" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D44" s="7"/>
-    </row>
-    <row r="46" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E44" s="1"/>
+      <c r="F44" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
+    </row>
+    <row r="46" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>41</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+      <c r="I46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B47" s="13"/>
       <c r="C47" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D47" s="12"/>
-      <c r="F47" s="0" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F47" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D48" s="12"/>
-      <c r="F48" s="0" t="s">
-        <v>43</v>
-      </c>
+      <c r="E48" s="1"/>
+      <c r="F48" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H48" s="0"/>
+      <c r="I48" s="0"/>
     </row>
     <row r="50" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C50" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D50" s="7"/>
+    </row>
+    <row r="51" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="0"/>
+      <c r="G51" s="0"/>
+      <c r="H51" s="0"/>
+      <c r="I51" s="0"/>
     </row>
     <row r="52" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="53" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>47</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B53" s="6"/>
       <c r="C53" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D53" s="7"/>
-    </row>
-    <row r="54" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>48</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B54" s="6"/>
       <c r="C54" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D54" s="7"/>
-    </row>
-    <row r="55" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+    </row>
+    <row r="55" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>49</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B55" s="1"/>
       <c r="C55" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D55" s="7"/>
-    </row>
-    <row r="56" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E55" s="1"/>
+      <c r="F55" s="0"/>
+      <c r="G55" s="0"/>
+      <c r="H55" s="0"/>
+      <c r="I55" s="0"/>
+    </row>
+    <row r="56" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>50</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B56" s="1"/>
       <c r="C56" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D56" s="7"/>
-    </row>
-    <row r="57" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E56" s="1"/>
+      <c r="F56" s="0"/>
+      <c r="G56" s="0"/>
+      <c r="H56" s="0"/>
+      <c r="I56" s="0"/>
+    </row>
+    <row r="57" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>51</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B57" s="6"/>
       <c r="C57" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D57" s="7"/>
-    </row>
-    <row r="58" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
+      <c r="H57" s="6"/>
+      <c r="I57" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B58" s="6"/>
       <c r="C58" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D58" s="7"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C59" s="7" t="n">
         <v>1</v>
@@ -1113,24 +1292,40 @@
     </row>
     <row r="60" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C60" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="7"/>
     </row>
-    <row r="63" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="0"/>
+      <c r="G61" s="0"/>
+      <c r="H61" s="0"/>
+      <c r="I61" s="0"/>
+    </row>
+    <row r="63" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
     </row>
     <row r="64" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>3</v>
@@ -1139,7 +1334,7 @@
     </row>
     <row r="65" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C65" s="7" t="n">
         <v>1</v>
@@ -1148,7 +1343,7 @@
     </row>
     <row r="66" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B66" s="9"/>
       <c r="C66" s="7"/>
@@ -1156,7 +1351,7 @@
     </row>
     <row r="67" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C67" s="7" t="n">
         <v>1</v>
@@ -1165,7 +1360,7 @@
     </row>
     <row r="68" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>1</v>
@@ -1174,7 +1369,7 @@
     </row>
     <row r="69" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C69" s="7" t="n">
         <v>1</v>
@@ -1183,7 +1378,7 @@
     </row>
     <row r="70" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>1</v>
@@ -1192,32 +1387,44 @@
     </row>
     <row r="71" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C71" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="D71" s="7"/>
     </row>
-    <row r="72" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>64</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="B72" s="1"/>
       <c r="C72" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="D72" s="7"/>
-    </row>
-    <row r="74" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E72" s="1"/>
+      <c r="F72" s="0"/>
+      <c r="G72" s="0"/>
+      <c r="H72" s="0"/>
+      <c r="I72" s="0"/>
+    </row>
+    <row r="74" s="15" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>65</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="B74" s="6"/>
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
-    </row>
-    <row r="76" s="15" customFormat="true" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E74" s="6"/>
+      <c r="F74" s="6"/>
+      <c r="G74" s="6"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
+    </row>
+    <row r="76" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B76" s="15" t="n">
         <f aca="false">IF(MIN(B9:B19)=1,SUM(B25:B74),0)</f>
@@ -1231,6 +1438,11 @@
         <f aca="false">SUM(D25:D74)</f>
         <v>2</v>
       </c>
+      <c r="E76" s="15"/>
+      <c r="F76" s="15"/>
+      <c r="G76" s="15"/>
+      <c r="H76" s="15"/>
+      <c r="I76" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B9:B19">

</xml_diff>

<commit_message>
Adds readme.md Final integration Updates checklist
</commit_message>
<xml_diff>
--- a/documentation/reports/checklist.xlsx
+++ b/documentation/reports/checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="66">
   <si>
     <t xml:space="preserve">Checklist Tourplanner Exam - Final Hand-In</t>
   </si>
@@ -94,24 +94,9 @@
     <t xml:space="preserve">GUI in general</t>
   </si>
   <si>
-    <t xml:space="preserve">Frontend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F. Impl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B. Impl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Correct data binding between UI elements and view model properties</t>
   </si>
   <si>
-    <t xml:space="preserve">x</t>
-  </si>
-  <si>
     <t xml:space="preserve">UI responds to window size changes</t>
   </si>
   <si>
@@ -130,9 +115,6 @@
     <t xml:space="preserve">Tours have computed attributes</t>
   </si>
   <si>
-    <t xml:space="preserve">frontend</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tour Details show all tour attributes of a selected tour and also the map image</t>
   </si>
   <si>
@@ -155,6 +137,9 @@
   </si>
   <si>
     <t xml:space="preserve">Search performs full-text search in Tours, Tour Logs and computed attributes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">only partialy implemented (search tour logs)</t>
   </si>
   <si>
     <t xml:space="preserve">List of Tours according to current search</t>
@@ -714,7 +699,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="18.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="48.41"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -865,70 +851,47 @@
       <c r="A24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="25" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H25" s="0" t="s">
-        <v>29</v>
-      </c>
+      <c r="F25" s="6"/>
+      <c r="H25" s="1"/>
       <c r="I25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
     </row>
-    <row r="27" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F27" s="6"/>
       <c r="G27" s="1"/>
-      <c r="H27" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -941,7 +904,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="10" t="n">
@@ -950,30 +913,22 @@
       <c r="D30" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
-      <c r="F31" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12" t="n">
@@ -982,16 +937,11 @@
       <c r="D32" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="12" t="n">
@@ -1000,62 +950,52 @@
       <c r="D33" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="E33" s="1"/>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
     </row>
     <row r="34" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F34" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="12"/>
-      <c r="F37" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D37" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="1"/>
+      <c r="H37" s="0"/>
+      <c r="I37" s="0"/>
     </row>
     <row r="38" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B38" s="9"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
-      <c r="G38" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="G38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C39" s="7" t="n">
         <v>1</v>
@@ -1063,28 +1003,35 @@
       <c r="D39" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E39" s="0"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F40" s="6"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
     </row>
+    <row r="41" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="0"/>
+      <c r="G41" s="0"/>
+      <c r="H41" s="0"/>
+      <c r="I41" s="0"/>
+    </row>
     <row r="42" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -1095,24 +1042,24 @@
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
     </row>
-    <row r="43" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>44</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B43" s="1"/>
       <c r="C43" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D43" s="7"/>
-      <c r="F43" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="E43" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H43" s="0"/>
+      <c r="I43" s="0"/>
     </row>
     <row r="44" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B44" s="1"/>
       <c r="C44" s="7" t="n">
@@ -1120,18 +1067,23 @@
       </c>
       <c r="D44" s="7"/>
       <c r="E44" s="1"/>
-      <c r="F44" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
     </row>
+    <row r="45" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="0"/>
+      <c r="G45" s="0"/>
+      <c r="H45" s="0"/>
+      <c r="I45" s="0"/>
+    </row>
     <row r="46" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -1144,67 +1096,81 @@
     </row>
     <row r="47" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B47" s="13"/>
       <c r="C47" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D47" s="12"/>
-      <c r="F47" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D47" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="6"/>
+      <c r="G47" s="6"/>
     </row>
     <row r="48" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D48" s="12"/>
+      <c r="D48" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="E48" s="1"/>
-      <c r="F48" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G48" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
-    <row r="50" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="0"/>
+      <c r="G49" s="0"/>
+      <c r="H49" s="0"/>
+      <c r="I49" s="0"/>
+    </row>
+    <row r="50" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>49</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B50" s="6"/>
       <c r="C50" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D50" s="7"/>
-    </row>
-    <row r="51" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>50</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="n">
@@ -1219,62 +1185,50 @@
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
     </row>
-    <row r="54" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B54" s="6"/>
+        <v>47</v>
+      </c>
       <c r="C54" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="7"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-    </row>
-    <row r="55" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D54" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B55" s="1"/>
+        <v>48</v>
+      </c>
       <c r="C55" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E55" s="1"/>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
-      <c r="H55" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="H55" s="1"/>
       <c r="I55" s="1"/>
     </row>
-    <row r="56" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B56" s="1"/>
+        <v>49</v>
+      </c>
       <c r="C56" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D56" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E56" s="1"/>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
-      <c r="H56" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="H56" s="1"/>
       <c r="I56" s="1"/>
     </row>
     <row r="57" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="n">
@@ -1291,7 +1245,7 @@
     </row>
     <row r="58" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="n">
@@ -1308,28 +1262,27 @@
     </row>
     <row r="59" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C59" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D59" s="7"/>
+      <c r="D59" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C60" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="7"/>
-    </row>
-    <row r="61" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
+      <c r="D60" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
@@ -1337,7 +1290,7 @@
     </row>
     <row r="63" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -1350,93 +1303,119 @@
     </row>
     <row r="64" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D64" s="7"/>
-    </row>
-    <row r="65" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D64" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>61</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B65" s="1"/>
       <c r="C65" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D65" s="7"/>
+      <c r="D65" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="1"/>
+      <c r="F65" s="0"/>
+      <c r="G65" s="0"/>
+      <c r="H65" s="0"/>
+      <c r="I65" s="0"/>
     </row>
     <row r="66" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B66" s="9"/>
       <c r="C66" s="7"/>
       <c r="D66" s="7"/>
     </row>
-    <row r="67" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" s="15" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>63</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B67" s="1"/>
       <c r="C67" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D67" s="7"/>
+      <c r="D67" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="1"/>
+      <c r="F67" s="0"/>
+      <c r="G67" s="0"/>
+      <c r="H67" s="0"/>
+      <c r="I67" s="0"/>
     </row>
     <row r="68" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D68" s="7"/>
+      <c r="D68" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C69" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D69" s="7"/>
+      <c r="D69" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D70" s="7"/>
+      <c r="D70" s="7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C71" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="D71" s="7"/>
-    </row>
-    <row r="72" s="6" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D71" s="7" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B72" s="1"/>
+        <v>63</v>
+      </c>
       <c r="C72" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="D72" s="7"/>
-      <c r="E72" s="1"/>
+      <c r="D72" s="7" t="n">
+        <v>0.5</v>
+      </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
       <c r="I72" s="1"/>
     </row>
-    <row r="74" s="15" customFormat="true" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7"/>
@@ -1449,7 +1428,7 @@
     </row>
     <row r="76" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="15" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B76" s="15" t="n">
         <f aca="false">IF(MIN(B9:B19)=1,SUM(B25:B74),0)</f>
@@ -1461,7 +1440,7 @@
       </c>
       <c r="D76" s="15" t="n">
         <f aca="false">SUM(D25:D74)</f>
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="E76" s="15"/>
       <c r="F76" s="15"/>

</xml_diff>